<commit_message>
run 2024 investment scenario
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/01_paper_IAEE/inputs_IAEE_2025_run_2024_inv.xlsx
+++ b/01_data/01_input_data/02_processed/01_paper_IAEE/inputs_IAEE_2025_run_2024_inv.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\01_paper_IAEE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFB33836-EFBC-41E7-8760-7A1107347CC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B72D68F5-0FF9-499F-B2D1-929F26C994ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5207,7 +5207,7 @@
         <v>849.02859328995112</v>
       </c>
       <c r="G2">
-        <v>1</v>
+        <v>252.48678804308389</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -5236,7 +5236,7 @@
         <v>668.70501516121294</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>198.86159637110859</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -5265,7 +5265,7 @@
         <v>238.73631348788709</v>
       </c>
       <c r="G4">
-        <v>1</v>
+        <v>70.996154261695125</v>
       </c>
       <c r="H4">
         <v>0</v>
@@ -5294,7 +5294,7 @@
         <v>663.92585689960322</v>
       </c>
       <c r="G5">
-        <v>1</v>
+        <v>197.44035528622641</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -5323,7 +5323,7 @@
         <v>608.75021221036775</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>181.0320488806565</v>
       </c>
       <c r="H6">
         <v>0</v>
@@ -5352,7 +5352,7 @@
         <v>522.98583818364546</v>
       </c>
       <c r="G7">
-        <v>1</v>
+        <v>155.5271701313755</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -5381,7 +5381,7 @@
         <v>1300.0820439640061</v>
       </c>
       <c r="G8">
-        <v>1</v>
+        <v>386.62247899212713</v>
       </c>
       <c r="H8">
         <v>0</v>
@@ -5410,7 +5410,7 @@
         <v>548.43418351199762</v>
       </c>
       <c r="G9">
-        <v>1</v>
+        <v>163.09507894357321</v>
       </c>
       <c r="H9">
         <v>0</v>
@@ -5439,7 +5439,7 @@
         <v>2452.8956460783979</v>
       </c>
       <c r="G10">
-        <v>1</v>
+        <v>729.449806493967</v>
       </c>
       <c r="H10">
         <v>0</v>
@@ -5468,7 +5468,7 @@
         <v>1496.537660139963</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>445.04506677457721</v>
       </c>
       <c r="H11">
         <v>0</v>
@@ -5497,7 +5497,7 @@
         <v>324.59315439382618</v>
       </c>
       <c r="G12">
-        <v>1</v>
+        <v>96.528531101756968</v>
       </c>
       <c r="H12">
         <v>0</v>
@@ -5526,7 +5526,7 @@
         <v>348.34127495826192</v>
       </c>
       <c r="G13">
-        <v>1</v>
+        <v>103.5908217369165</v>
       </c>
       <c r="H13">
         <v>0</v>
@@ -5555,7 +5555,7 @@
         <v>818.47852582492351</v>
       </c>
       <c r="G14">
-        <v>1</v>
+        <v>243.40171308835841</v>
       </c>
       <c r="H14">
         <v>0</v>
@@ -5584,7 +5584,7 @@
         <v>2635.6088276270129</v>
       </c>
       <c r="G15">
-        <v>1</v>
+        <v>783.7856259315439</v>
       </c>
       <c r="H15">
         <v>0</v>
@@ -5613,7 +5613,7 @@
         <v>1845.982111336245</v>
       </c>
       <c r="G16">
-        <v>1</v>
+        <v>548.96395452385684</v>
       </c>
       <c r="H16">
         <v>0</v>
@@ -5642,7 +5642,7 @@
         <v>1022.460605388272</v>
       </c>
       <c r="G17">
-        <v>1</v>
+        <v>304.06254417736523</v>
       </c>
       <c r="H17">
         <v>0</v>
@@ -5671,7 +5671,7 @@
         <v>772.41845598916768</v>
       </c>
       <c r="G18">
-        <v>1</v>
+        <v>229.70422494510751</v>
       </c>
       <c r="H18">
         <v>0</v>
@@ -5700,7 +5700,7 @@
         <v>1058.6299231685789</v>
       </c>
       <c r="G19">
-        <v>1</v>
+        <v>314.81868942881317</v>
       </c>
       <c r="H19">
         <v>0</v>
@@ -5729,7 +5729,7 @@
         <v>238.73631348788709</v>
       </c>
       <c r="G20">
-        <v>1</v>
+        <v>70.996154261695125</v>
       </c>
       <c r="H20">
         <v>0</v>
@@ -5758,7 +5758,7 @@
         <v>554.29660486213618</v>
       </c>
       <c r="G21">
-        <v>1</v>
+        <v>164.8384642059188</v>
       </c>
       <c r="H21">
         <v>0</v>
@@ -5787,7 +5787,7 @@
         <v>1561.553620994126</v>
       </c>
       <c r="G22">
-        <v>1</v>
+        <v>464.37971728851619</v>
       </c>
       <c r="H22">
         <v>0</v>
@@ -5816,7 +5816,7 @@
         <v>655.82189631712072</v>
       </c>
       <c r="G23">
-        <v>1</v>
+        <v>195.0303740511186</v>
       </c>
       <c r="H23">
         <v>0</v>
@@ -5845,7 +5845,7 @@
         <v>735.1327792936105</v>
       </c>
       <c r="G24">
-        <v>1</v>
+        <v>218.61609337536299</v>
       </c>
       <c r="H24">
         <v>0</v>
@@ -5874,7 +5874,7 @@
         <v>589.26805934605818</v>
       </c>
       <c r="G25">
-        <v>1</v>
+        <v>175.23838511037869</v>
       </c>
       <c r="H25">
         <v>0</v>
@@ -5903,7 +5903,7 @@
         <v>1496.537660139963</v>
       </c>
       <c r="G26">
-        <v>1</v>
+        <v>445.04506677457721</v>
       </c>
       <c r="H26">
         <v>0</v>
@@ -5932,7 +5932,7 @@
         <v>1085.4804188182641</v>
       </c>
       <c r="G27">
-        <v>1</v>
+        <v>322.80357410470373</v>
       </c>
       <c r="H27">
         <v>0</v>
@@ -5961,7 +5961,7 @@
         <v>655.82189631712072</v>
       </c>
       <c r="G28">
-        <v>1</v>
+        <v>195.0303740511186</v>
       </c>
       <c r="H28">
         <v>0</v>
@@ -5990,7 +5990,7 @@
         <v>293.03385025058509</v>
       </c>
       <c r="G29">
-        <v>1</v>
+        <v>87.143326175825223</v>
       </c>
       <c r="H29">
         <v>0</v>
@@ -6019,7 +6019,7 @@
         <v>818.47852582492351</v>
       </c>
       <c r="G30">
-        <v>1</v>
+        <v>243.40171308835841</v>
       </c>
       <c r="H30">
         <v>0</v>
@@ -6048,7 +6048,7 @@
         <v>515.80069466505029</v>
       </c>
       <c r="G31">
-        <v>1</v>
+        <v>153.39042959875229</v>
       </c>
       <c r="H31">
         <v>0</v>
@@ -6077,7 +6077,7 @@
         <v>1527.199701791101</v>
       </c>
       <c r="G32">
-        <v>1</v>
+        <v>454.16344096423802</v>
       </c>
       <c r="H32">
         <v>0</v>
@@ -6106,7 +6106,7 @@
         <v>608.75021221036775</v>
       </c>
       <c r="G33">
-        <v>1</v>
+        <v>181.0320488806565</v>
       </c>
       <c r="H33">
         <v>0</v>
@@ -6135,7 +6135,7 @@
         <v>570.0535608755265</v>
       </c>
       <c r="G34">
-        <v>1</v>
+        <v>169.52431724384871</v>
       </c>
       <c r="H34">
         <v>0</v>
@@ -6164,7 +6164,7 @@
         <v>308.62014069696289</v>
       </c>
       <c r="G35">
-        <v>1</v>
+        <v>91.778426151743929</v>
       </c>
       <c r="H35">
         <v>0</v>
@@ -6193,7 +6193,7 @@
         <v>1279.0874423010839</v>
       </c>
       <c r="G36">
-        <v>1</v>
+        <v>380.37903845077301</v>
       </c>
       <c r="H36">
         <v>0</v>
@@ -6222,7 +6222,7 @@
         <v>1578.4655807813269</v>
       </c>
       <c r="G37">
-        <v>1</v>
+        <v>469.40904897408171</v>
       </c>
       <c r="H37">
         <v>0</v>
@@ -6251,7 +6251,7 @@
         <v>802.2610733299972</v>
       </c>
       <c r="G38">
-        <v>1</v>
+        <v>238.5789161613215</v>
       </c>
       <c r="H38">
         <v>0</v>
@@ -6280,7 +6280,7 @@
         <v>968.14625408077427</v>
       </c>
       <c r="G39">
-        <v>1</v>
+        <v>287.91037190112422</v>
       </c>
       <c r="H39">
         <v>0</v>
@@ -6309,7 +6309,7 @@
         <v>289.20816151374652</v>
       </c>
       <c r="G40">
-        <v>1</v>
+        <v>86.005630851014047</v>
       </c>
       <c r="H40">
         <v>0</v>
@@ -6338,7 +6338,7 @@
         <v>928.64894808112615</v>
       </c>
       <c r="G41">
-        <v>1</v>
+        <v>276.16453906696393</v>
       </c>
       <c r="H41">
         <v>0</v>
@@ -6367,7 +6367,7 @@
         <v>1646.127432515166</v>
       </c>
       <c r="G42">
-        <v>1</v>
+        <v>1000000</v>
       </c>
       <c r="H42">
         <v>0</v>
@@ -6396,7 +6396,7 @@
         <v>649.46853875803151</v>
       </c>
       <c r="G43">
-        <v>1</v>
+        <v>193.14099263798181</v>
       </c>
       <c r="H43">
         <v>0</v>
@@ -6425,7 +6425,7 @@
         <v>2379.117070154653</v>
       </c>
       <c r="G44">
-        <v>1</v>
+        <v>707.50930200613095</v>
       </c>
       <c r="H44">
         <v>0</v>
@@ -6454,7 +6454,7 @@
         <v>589.26805934605818</v>
       </c>
       <c r="G45">
-        <v>1</v>
+        <v>175.23838511037869</v>
       </c>
       <c r="H45">
         <v>0</v>
@@ -6483,7 +6483,7 @@
         <v>308.62014069696289</v>
       </c>
       <c r="G46">
-        <v>1</v>
+        <v>91.778426151743929</v>
       </c>
       <c r="H46">
         <v>0</v>
@@ -6512,7 +6512,7 @@
         <v>1300.0820439640061</v>
       </c>
       <c r="G47">
-        <v>1</v>
+        <v>386.62247899212713</v>
       </c>
       <c r="H47">
         <v>0</v>
@@ -6541,7 +6541,7 @@
         <v>687.19761214976381</v>
       </c>
       <c r="G48">
-        <v>1</v>
+        <v>204.36098290898909</v>
       </c>
       <c r="H48">
         <v>0</v>
@@ -6570,7 +6570,7 @@
         <v>679.24293689571005</v>
       </c>
       <c r="G49">
-        <v>1</v>
+        <v>201.9953966134332</v>
       </c>
       <c r="H49">
         <v>0</v>
@@ -6599,7 +6599,7 @@
         <v>1279.0874423010839</v>
       </c>
       <c r="G50">
-        <v>1</v>
+        <v>380.37903845077301</v>
       </c>
       <c r="H50">
         <v>0</v>
@@ -6628,7 +6628,7 @@
         <v>968.14625408077427</v>
       </c>
       <c r="G51">
-        <v>1</v>
+        <v>287.91037190112422</v>
       </c>
       <c r="H51">
         <v>0</v>
@@ -6657,7 +6657,7 @@
         <v>749.61752413264298</v>
       </c>
       <c r="G52">
-        <v>1</v>
+        <v>222.9236122609866</v>
       </c>
       <c r="H52">
         <v>0</v>
@@ -6686,7 +6686,7 @@
         <v>653.9464650405971</v>
       </c>
       <c r="G53">
-        <v>1</v>
+        <v>194.47265241141491</v>
       </c>
       <c r="H53">
         <v>0</v>
@@ -6715,7 +6715,7 @@
         <v>324.59315439382618</v>
       </c>
       <c r="G54">
-        <v>1</v>
+        <v>96.528531101756968</v>
       </c>
       <c r="H54">
         <v>0</v>
@@ -6744,7 +6744,7 @@
         <v>488.85694823775901</v>
       </c>
       <c r="G55">
-        <v>1</v>
+        <v>145.37781371391739</v>
       </c>
       <c r="H55">
         <v>0</v>
@@ -6773,7 +6773,7 @@
         <v>1568.236027931837</v>
       </c>
       <c r="G56">
-        <v>1</v>
+        <v>466.36695243870309</v>
       </c>
       <c r="H56">
         <v>0</v>
@@ -6802,7 +6802,7 @@
         <v>1032.4558391947651</v>
       </c>
       <c r="G57">
-        <v>1</v>
+        <v>307.03495818024572</v>
       </c>
       <c r="H57">
         <v>0</v>
@@ -6831,7 +6831,7 @@
         <v>709.04398925426131</v>
       </c>
       <c r="G58">
-        <v>1</v>
+        <v>210.85772710475121</v>
       </c>
       <c r="H58">
         <v>0</v>
@@ -6860,7 +6860,7 @@
         <v>1058.6299231685789</v>
       </c>
       <c r="G59">
-        <v>1</v>
+        <v>314.81868942881317</v>
       </c>
       <c r="H59">
         <v>0</v>
@@ -6889,7 +6889,7 @@
         <v>999999</v>
       </c>
       <c r="G60">
-        <v>1</v>
+        <v>1000000</v>
       </c>
       <c r="H60">
         <v>0</v>
@@ -6918,7 +6918,7 @@
         <v>644.52310193987068</v>
       </c>
       <c r="G61">
-        <v>1</v>
+        <v>191.67030311402959</v>
       </c>
       <c r="H61">
         <v>0</v>
@@ -6947,7 +6947,7 @@
         <v>1589.018295636323</v>
       </c>
       <c r="G62">
-        <v>1</v>
+        <v>1000000</v>
       </c>
       <c r="H62">
         <v>0</v>
@@ -6976,7 +6976,7 @@
         <v>749.61752413264298</v>
       </c>
       <c r="G63">
-        <v>1</v>
+        <v>222.9236122609866</v>
       </c>
       <c r="H63">
         <v>0</v>
@@ -7005,7 +7005,7 @@
         <v>644.52310193987068</v>
       </c>
       <c r="G64">
-        <v>1</v>
+        <v>191.67030311402959</v>
       </c>
       <c r="H64">
         <v>0</v>
@@ -7034,7 +7034,7 @@
         <v>849.02859328995112</v>
       </c>
       <c r="G65">
-        <v>1</v>
+        <v>252.48678804308389</v>
       </c>
       <c r="H65">
         <v>0</v>
@@ -7063,7 +7063,7 @@
         <v>687.19761214976381</v>
       </c>
       <c r="G66">
-        <v>1</v>
+        <v>204.36098290898909</v>
       </c>
       <c r="H66">
         <v>0</v>
@@ -7092,7 +7092,7 @@
         <v>348.34127495826192</v>
       </c>
       <c r="G67">
-        <v>1</v>
+        <v>103.5908217369165</v>
       </c>
       <c r="H67">
         <v>0</v>
@@ -7121,7 +7121,7 @@
         <v>1439.4957302840339</v>
       </c>
       <c r="G68">
-        <v>1</v>
+        <v>428.08175862815312</v>
       </c>
       <c r="H68">
         <v>0</v>
@@ -7150,7 +7150,7 @@
         <v>907.81699800561239</v>
       </c>
       <c r="G69">
-        <v>1</v>
+        <v>269.96946836521192</v>
       </c>
       <c r="H69">
         <v>0</v>
@@ -7179,7 +7179,7 @@
         <v>568.81179966066486</v>
       </c>
       <c r="G70">
-        <v>1</v>
+        <v>169.15503839607521</v>
       </c>
       <c r="H70">
         <v>0</v>
@@ -7208,7 +7208,7 @@
         <v>999999</v>
       </c>
       <c r="G71">
-        <v>1</v>
+        <v>1000000</v>
       </c>
       <c r="H71">
         <v>0</v>
@@ -7237,7 +7237,7 @@
         <v>999999</v>
       </c>
       <c r="G72">
-        <v>1</v>
+        <v>1000000</v>
       </c>
       <c r="H72">
         <v>0</v>
@@ -7266,7 +7266,7 @@
         <v>1439.4957302840339</v>
       </c>
       <c r="G73">
-        <v>1</v>
+        <v>428.08175862815312</v>
       </c>
       <c r="H73">
         <v>0</v>
@@ -7295,7 +7295,7 @@
         <v>289.20816151374652</v>
       </c>
       <c r="G74">
-        <v>1</v>
+        <v>86.005630851014047</v>
       </c>
       <c r="H74">
         <v>0</v>
@@ -7324,7 +7324,7 @@
         <v>709.04398925426131</v>
       </c>
       <c r="G75">
-        <v>1</v>
+        <v>210.85772710475121</v>
       </c>
       <c r="H75">
         <v>0</v>
@@ -7353,7 +7353,7 @@
         <v>999999</v>
       </c>
       <c r="G76">
-        <v>1</v>
+        <v>1000000</v>
       </c>
       <c r="H76">
         <v>0</v>
@@ -7382,7 +7382,7 @@
         <v>554.29660486213618</v>
       </c>
       <c r="G77">
-        <v>1</v>
+        <v>164.8384642059188</v>
       </c>
       <c r="H77">
         <v>0</v>
@@ -7411,7 +7411,7 @@
         <v>2521.4020294179322</v>
       </c>
       <c r="G78">
-        <v>1</v>
+        <v>1000000</v>
       </c>
       <c r="H78">
         <v>0</v>
@@ -7440,7 +7440,7 @@
         <v>1032.4558391947651</v>
       </c>
       <c r="G79">
-        <v>1</v>
+        <v>307.03495818024572</v>
       </c>
       <c r="H79">
         <v>0</v>
@@ -7469,7 +7469,7 @@
         <v>584.70651753259665</v>
       </c>
       <c r="G80">
-        <v>1</v>
+        <v>173.8818594879115</v>
       </c>
       <c r="H80">
         <v>0</v>
@@ -7498,7 +7498,7 @@
         <v>928.64894808112615</v>
       </c>
       <c r="G81">
-        <v>1</v>
+        <v>276.16453906696393</v>
       </c>
       <c r="H81">
         <v>0</v>
@@ -7527,7 +7527,7 @@
         <v>1120.4319208210959</v>
       </c>
       <c r="G82">
-        <v>1</v>
+        <v>333.19756147770909</v>
       </c>
       <c r="H82">
         <v>0</v>
@@ -7556,7 +7556,7 @@
         <v>6330.2807560755737</v>
       </c>
       <c r="G83">
-        <v>1</v>
+        <v>1882.5187610220189</v>
       </c>
       <c r="H83">
         <v>0</v>
@@ -7585,7 +7585,7 @@
         <v>934.38709794225724</v>
       </c>
       <c r="G84">
-        <v>1</v>
+        <v>277.87096808383927</v>
       </c>
       <c r="H84">
         <v>0</v>
@@ -7614,7 +7614,7 @@
         <v>515.80069466505029</v>
       </c>
       <c r="G85">
-        <v>1</v>
+        <v>153.39042959875229</v>
       </c>
       <c r="H85">
         <v>0</v>
@@ -7643,7 +7643,7 @@
         <v>584.70651753259665</v>
       </c>
       <c r="G86">
-        <v>1</v>
+        <v>173.8818594879115</v>
       </c>
       <c r="H86">
         <v>0</v>
@@ -7672,7 +7672,7 @@
         <v>679.24293689571005</v>
       </c>
       <c r="G87">
-        <v>1</v>
+        <v>201.9953966134332</v>
       </c>
       <c r="H87">
         <v>0</v>
@@ -7701,7 +7701,7 @@
         <v>542.43529941219504</v>
       </c>
       <c r="G88">
-        <v>1</v>
+        <v>161.31111196039689</v>
       </c>
       <c r="H88">
         <v>0</v>
@@ -7730,7 +7730,7 @@
         <v>649.46853875803151</v>
       </c>
       <c r="G89">
-        <v>1</v>
+        <v>193.14099263798181</v>
       </c>
       <c r="H89">
         <v>0</v>
@@ -7759,7 +7759,7 @@
         <v>1673.064111521544</v>
       </c>
       <c r="G90">
-        <v>1</v>
+        <v>1000000</v>
       </c>
       <c r="H90">
         <v>0</v>
@@ -7788,7 +7788,7 @@
         <v>735.1327792936105</v>
       </c>
       <c r="G91">
-        <v>1</v>
+        <v>218.61609337536299</v>
       </c>
       <c r="H91">
         <v>0</v>
@@ -7817,7 +7817,7 @@
         <v>6046.2734369221553</v>
       </c>
       <c r="G92">
-        <v>1</v>
+        <v>1798.0597729967651</v>
       </c>
       <c r="H92">
         <v>0</v>
@@ -7846,7 +7846,7 @@
         <v>999999</v>
       </c>
       <c r="G93">
-        <v>1</v>
+        <v>1000000</v>
       </c>
       <c r="H93">
         <v>0</v>
@@ -7875,7 +7875,7 @@
         <v>792.519650598206</v>
       </c>
       <c r="G94">
-        <v>1</v>
+        <v>235.68198129250979</v>
       </c>
       <c r="H94">
         <v>0</v>
@@ -7904,7 +7904,7 @@
         <v>1029.314499712772</v>
       </c>
       <c r="G95">
-        <v>1</v>
+        <v>306.10077678490791</v>
       </c>
       <c r="H95">
         <v>0</v>
@@ -7933,7 +7933,7 @@
         <v>293.03385025058509</v>
       </c>
       <c r="G96">
-        <v>1</v>
+        <v>87.143326175825223</v>
       </c>
       <c r="H96">
         <v>0</v>
@@ -7962,7 +7962,7 @@
         <v>293.41708096429733</v>
       </c>
       <c r="G97">
-        <v>1</v>
+        <v>87.25729252837138</v>
       </c>
       <c r="H97">
         <v>0</v>
@@ -7991,7 +7991,7 @@
         <v>681.90695066602268</v>
       </c>
       <c r="G98">
-        <v>1</v>
+        <v>202.78762939037941</v>
       </c>
       <c r="H98">
         <v>0</v>
@@ -8020,7 +8020,7 @@
         <v>410.42142246837989</v>
       </c>
       <c r="G99">
-        <v>1</v>
+        <v>122.0524108635357</v>
       </c>
       <c r="H99">
         <v>0</v>
@@ -8049,7 +8049,7 @@
         <v>668.70501516121294</v>
       </c>
       <c r="G100">
-        <v>1</v>
+        <v>198.86159637110859</v>
       </c>
       <c r="H100">
         <v>0</v>
@@ -8078,7 +8078,7 @@
         <v>945.089569229208</v>
       </c>
       <c r="G101">
-        <v>1</v>
+        <v>281.0537025885684</v>
       </c>
       <c r="H101">
         <v>0</v>
@@ -8107,7 +8107,7 @@
         <v>1736.696056306987</v>
       </c>
       <c r="G102">
-        <v>1</v>
+        <v>1000000</v>
       </c>
       <c r="H102">
         <v>0</v>
@@ -8136,7 +8136,7 @@
         <v>3131.085096797216</v>
       </c>
       <c r="G103">
-        <v>1</v>
+        <v>1000000</v>
       </c>
       <c r="H103">
         <v>0</v>
@@ -8165,7 +8165,7 @@
         <v>2312.4197737153231</v>
       </c>
       <c r="G104">
-        <v>1</v>
+        <v>687.67465063842064</v>
       </c>
       <c r="H104">
         <v>0</v>
@@ -8194,7 +8194,7 @@
         <v>999999</v>
       </c>
       <c r="G105">
-        <v>1</v>
+        <v>1000000</v>
       </c>
       <c r="H105">
         <v>0</v>
@@ -8223,7 +8223,7 @@
         <v>934.38709794225724</v>
       </c>
       <c r="G106">
-        <v>1</v>
+        <v>277.87096808383927</v>
       </c>
       <c r="H106">
         <v>0</v>
@@ -8252,7 +8252,7 @@
         <v>802.2610733299972</v>
       </c>
       <c r="G107">
-        <v>1</v>
+        <v>238.5789161613215</v>
       </c>
       <c r="H107">
         <v>0</v>
@@ -8281,7 +8281,7 @@
         <v>1029.314499712772</v>
       </c>
       <c r="G108">
-        <v>1</v>
+        <v>306.10077678490791</v>
       </c>
       <c r="H108">
         <v>0</v>
@@ -8310,7 +8310,7 @@
         <v>1578.4655807813269</v>
       </c>
       <c r="G109">
-        <v>1</v>
+        <v>469.40904897408171</v>
       </c>
       <c r="H109">
         <v>0</v>
@@ -8339,7 +8339,7 @@
         <v>548.43418351199762</v>
       </c>
       <c r="G110">
-        <v>1</v>
+        <v>163.09507894357321</v>
       </c>
       <c r="H110">
         <v>0</v>
@@ -8368,7 +8368,7 @@
         <v>1085.4804188182641</v>
       </c>
       <c r="G111">
-        <v>1</v>
+        <v>322.80357410470373</v>
       </c>
       <c r="H111">
         <v>0</v>
@@ -8397,7 +8397,7 @@
         <v>772.41845598916768</v>
       </c>
       <c r="G112">
-        <v>1</v>
+        <v>229.70422494510751</v>
       </c>
       <c r="H112">
         <v>0</v>
@@ -8426,7 +8426,7 @@
         <v>1364.317119921996</v>
       </c>
       <c r="G113">
-        <v>1</v>
+        <v>405.7249075045641</v>
       </c>
       <c r="H113">
         <v>0</v>
@@ -8455,7 +8455,7 @@
         <v>3449.967874173466</v>
       </c>
       <c r="G114">
-        <v>1</v>
+        <v>1025.962275341657</v>
       </c>
       <c r="H114">
         <v>0</v>
@@ -8484,7 +8484,7 @@
         <v>907.81699800561239</v>
       </c>
       <c r="G115">
-        <v>1</v>
+        <v>269.96946836521192</v>
       </c>
       <c r="H115">
         <v>0</v>
@@ -8513,7 +8513,7 @@
         <v>522.98583818364546</v>
       </c>
       <c r="G116">
-        <v>1</v>
+        <v>155.5271701313755</v>
       </c>
       <c r="H116">
         <v>0</v>

</xml_diff>